<commit_message>
Bugfixes, added glutine table
</commit_message>
<xml_diff>
--- a/static/esempio_paziente_completo.xlsx
+++ b/static/esempio_paziente_completo.xlsx
@@ -711,11 +711,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="2" style="2" width="24.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="23.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="21.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="21.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="0" width="23.28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -775,6 +779,11 @@
       <c r="T3" s="7"/>
       <c r="U3" s="8"/>
       <c r="V3" s="9"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="8"/>
+      <c r="Y3" s="9"/>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="11"/>
     </row>
     <row r="4" s="26" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
@@ -801,6 +810,11 @@
       <c r="T4" s="17"/>
       <c r="U4" s="18"/>
       <c r="V4" s="19"/>
+      <c r="W4" s="17"/>
+      <c r="X4" s="18"/>
+      <c r="Y4" s="19"/>
+      <c r="Z4" s="20"/>
+      <c r="AA4" s="21"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
@@ -827,6 +841,11 @@
       <c r="T5" s="27"/>
       <c r="U5" s="28"/>
       <c r="V5" s="29"/>
+      <c r="W5" s="27"/>
+      <c r="X5" s="28"/>
+      <c r="Y5" s="29"/>
+      <c r="Z5" s="30"/>
+      <c r="AA5" s="31"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
@@ -853,6 +872,11 @@
       <c r="T6" s="27"/>
       <c r="U6" s="28"/>
       <c r="V6" s="29"/>
+      <c r="W6" s="27"/>
+      <c r="X6" s="28"/>
+      <c r="Y6" s="29"/>
+      <c r="Z6" s="30"/>
+      <c r="AA6" s="31"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="36" t="s">
@@ -879,6 +903,11 @@
       <c r="T7" s="27"/>
       <c r="U7" s="28"/>
       <c r="V7" s="29"/>
+      <c r="W7" s="27"/>
+      <c r="X7" s="28"/>
+      <c r="Y7" s="29"/>
+      <c r="Z7" s="30"/>
+      <c r="AA7" s="31"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
@@ -905,6 +934,11 @@
       <c r="T8" s="7"/>
       <c r="U8" s="8"/>
       <c r="V8" s="9"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
@@ -931,6 +965,11 @@
       <c r="T9" s="7"/>
       <c r="U9" s="8"/>
       <c r="V9" s="9"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="9"/>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
@@ -957,6 +996,11 @@
       <c r="T10" s="7"/>
       <c r="U10" s="8"/>
       <c r="V10" s="9"/>
+      <c r="W10" s="7"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="9"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
@@ -983,6 +1027,11 @@
       <c r="T11" s="7"/>
       <c r="U11" s="8"/>
       <c r="V11" s="9"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="9"/>
+      <c r="Z11" s="10"/>
+      <c r="AA11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -1009,6 +1058,11 @@
       <c r="T12" s="37"/>
       <c r="U12" s="38"/>
       <c r="V12" s="39"/>
+      <c r="W12" s="37"/>
+      <c r="X12" s="38"/>
+      <c r="Y12" s="39"/>
+      <c r="Z12" s="40"/>
+      <c r="AA12" s="41"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
@@ -1035,6 +1089,11 @@
       <c r="T13" s="46"/>
       <c r="U13" s="47"/>
       <c r="V13" s="48"/>
+      <c r="W13" s="46"/>
+      <c r="X13" s="47"/>
+      <c r="Y13" s="48"/>
+      <c r="Z13" s="49"/>
+      <c r="AA13" s="50"/>
     </row>
     <row r="14" s="64" customFormat="true" ht="51.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
@@ -1061,6 +1120,11 @@
       <c r="T14" s="55"/>
       <c r="U14" s="56"/>
       <c r="V14" s="57"/>
+      <c r="W14" s="55"/>
+      <c r="X14" s="56"/>
+      <c r="Y14" s="57"/>
+      <c r="Z14" s="58"/>
+      <c r="AA14" s="59"/>
     </row>
     <row r="15" s="64" customFormat="true" ht="24.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
@@ -1087,6 +1151,11 @@
       <c r="T15" s="65"/>
       <c r="U15" s="66"/>
       <c r="V15" s="67"/>
+      <c r="W15" s="65"/>
+      <c r="X15" s="66"/>
+      <c r="Y15" s="67"/>
+      <c r="Z15" s="68"/>
+      <c r="AA15" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1094,19 +1163,19 @@
     <mergeCell ref="B2:V2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B15 K15 T15" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B15 K15 T15 W15" type="list">
       <formula1>"Normale,DQ2.5 \ DQ2.5,DQ2.5 \ DQ2.2,DQ2.5 (cis),DQ2.5 (trans),DQ2.2 \ DQ2.2,DQ2.2 \ DQX,DQ8 \ DQ8,DQ8 \ DQX,DQ2.5 \ DQX,DQ2.5 \ DQ8,DQ7 \ DQX,DQ7 \ DQ7,DQ7 \ DQ2.2,DQ7 \ DQ8"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C15 L15 U15" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C15 L15 U15 X15" type="list">
       <formula1>"Normale,DQ2.5 \ DQ2.5,DQ2.5 \ DQ2.2,DQ2.5 (cis),DQ2.5 (trans),DQ2.2 \ DQ2.2,DQ2.2 \ DQX,DQ8 \ DQ8,DQ8 \ DQX,DQ2.5 \ DQX,DQ2.5 \ DQ8,DQ7 \ DQX,DQ7 \ DQ7,DQ7 \ DQ2.2,DQ7 \ DQ8"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D15:J15 M15:S15 V15" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D15:J15 M15:S15 V15 Y15:AA15" type="list">
       <formula1>"Normale,DQ2.5 \ DQ2.5,DQ2.5 \ DQ2.2,DQ2.5 (cis),DQ2.5 (trans),DQ2.2 \ DQ2.2,DQ2.2 \ DQX,DQ8 \ DQ8,DQ8 \ DQX,DQ2.5 \ DQX,DQ2.5 \ DQ8,DQ7 \ DQX,DQ7 \ DQ7,DQ7 \ DQ2.2,DQ7 \ DQ8"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B13:V13" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B13:AA13" type="list">
       <formula1>"Altamedica,Genessere,Braincare,Longevia,IkonFiumicino,IkonAcilia,IkonCasalPalocco"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>